<commit_message>
Inclusion de modelo para USA - Recupere datos extraídos de USA de compu local, extraje missing y entrene algunos modelos. Todo para poder probar cronjob de main_next_matches con una liga que tenga próximos partidos realmente (las otras ligas que tengo esta paradas). - En find_best: uso determine_comps() que ya tenia codeada en select_data.py
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
   <si>
     <t>id_country</t>
   </si>
@@ -239,6 +239,18 @@
   </si>
   <si>
     <t>(18, 32)</t>
+  </si>
+  <si>
+    <t>usa</t>
+  </si>
+  <si>
+    <t>[1671, 1672]</t>
+  </si>
+  <si>
+    <t>-0.05</t>
+  </si>
+  <si>
+    <t>(31, 32)</t>
   </si>
 </sst>
 </file>
@@ -248,7 +260,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy&quot;-&quot;mm&quot;-&quot;dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -263,6 +275,11 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -317,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -355,6 +372,18 @@
     </xf>
     <xf borderId="3" fillId="2" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1028,6 +1057,65 @@
       </c>
       <c r="V7" s="8"/>
     </row>
+    <row r="8">
+      <c r="A8" s="14">
+        <v>167.0</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="15">
+        <v>45460.0</v>
+      </c>
+      <c r="D8" s="14">
+        <v>4.0</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="16">
+        <v>45.0</v>
+      </c>
+      <c r="G8" s="16">
+        <v>3.0</v>
+      </c>
+      <c r="H8" s="16" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" s="16">
+        <v>10.0</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="N8" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="O8" s="15">
+        <v>45460.0</v>
+      </c>
+      <c r="P8" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="R8" s="17">
+        <v>0.0981</v>
+      </c>
+      <c r="S8" s="16">
+        <v>31.0</v>
+      </c>
+      <c r="T8" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>

</xml_diff>

<commit_message>
d_run como parametro en collect_predictions.py y arreglo error en usa en df_best_models
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -329,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -367,6 +367,9 @@
     </xf>
     <xf borderId="3" fillId="2" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -1063,16 +1066,16 @@
       <c r="B8" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="5">
-        <v>45460.0</v>
-      </c>
-      <c r="D8" s="14">
+      <c r="C8" s="14">
+        <v>45461.0</v>
+      </c>
+      <c r="D8" s="15">
         <v>690.0</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="16">
         <v>60.0</v>
       </c>
       <c r="G8" s="7">
@@ -1081,46 +1084,46 @@
       <c r="H8" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="J8" s="15" t="s">
+      <c r="J8" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="K8" s="15">
+      <c r="K8" s="16">
         <v>10.0</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>56</v>
       </c>
       <c r="M8" s="7"/>
-      <c r="N8" s="16" t="s">
+      <c r="N8" s="17" t="s">
         <v>35</v>
       </c>
       <c r="O8" s="5">
         <v>45461.0</v>
       </c>
-      <c r="P8" s="14" t="s">
+      <c r="P8" s="15" t="s">
         <v>46</v>
       </c>
       <c r="Q8" s="10">
         <f t="shared" si="3"/>
         <v>1.288548387</v>
       </c>
-      <c r="R8" s="17">
+      <c r="R8" s="18">
         <v>0.7989</v>
       </c>
       <c r="S8" s="7">
         <v>31.0</v>
       </c>
-      <c r="T8" s="16" t="s">
+      <c r="T8" s="17" t="s">
         <v>57</v>
       </c>
       <c r="U8" s="3">
         <f t="shared" si="2"/>
         <v>4.658598015</v>
       </c>
-      <c r="V8" s="18" t="s">
+      <c r="V8" s="19" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Extraigo missing de USA, evaluo modelos y selecciono nuevo modelo
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
   <si>
     <t>id_country</t>
   </si>
@@ -244,13 +244,16 @@
     <t>usa</t>
   </si>
   <si>
+    <t>0.7</t>
+  </si>
+  <si>
     <t>[1671, 1672]</t>
   </si>
   <si>
-    <t>(31, 37)</t>
-  </si>
-  <si>
-    <t>el mejor modelo segun el roi es el 219 pero es n_years=3, por lo que, entreno y se testeo con pocos partidos lo cual significa menos confiabilidad en sus rdos.</t>
+    <t>-0.05</t>
+  </si>
+  <si>
+    <t>(44, 20)</t>
   </si>
 </sst>
 </file>
@@ -1070,62 +1073,60 @@
         <v>45461.0</v>
       </c>
       <c r="D8" s="15">
-        <v>690.0</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>23</v>
+        <v>148.0</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>31</v>
       </c>
       <c r="F8" s="16">
-        <v>60.0</v>
+        <v>30.0</v>
       </c>
       <c r="G8" s="7">
         <v>3.0</v>
       </c>
-      <c r="H8" s="7" t="b">
-        <v>0</v>
+      <c r="H8" s="16" t="b">
+        <v>1</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="K8" s="16">
-        <v>10.0</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="K8" s="16"/>
       <c r="L8" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M8" s="7"/>
+        <v>57</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>34</v>
+      </c>
       <c r="N8" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="O8" s="5">
-        <v>45461.0</v>
+      <c r="O8" s="14">
+        <v>45463.0</v>
       </c>
       <c r="P8" s="15" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="Q8" s="10">
         <f t="shared" si="3"/>
-        <v>1.288548387</v>
+        <v>1.351106848</v>
       </c>
       <c r="R8" s="18">
-        <v>0.7989</v>
-      </c>
-      <c r="S8" s="7">
-        <v>31.0</v>
+        <v>1.18897402636724</v>
+      </c>
+      <c r="S8" s="16">
+        <v>44.0</v>
       </c>
       <c r="T8" s="17" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="U8" s="3">
         <f t="shared" si="2"/>
-        <v>4.658598015</v>
-      </c>
-      <c r="V8" s="19" t="s">
-        <v>58</v>
-      </c>
+        <v>4.884770913</v>
+      </c>
+      <c r="V8" s="19"/>
     </row>
   </sheetData>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
Soluciono problema en integracion de jugadores en df_integrated_missing
En scraper_flashscore.py:
- Descubri que no estaba extrayendo bien el id de un jugador de su url  tras el reciente cambio HTML de Flashscore. Actualizo la forma de extraer id del equipo/player de url y del nombre.

Data:
1. Vuelvo a extraer missing de todos los paises. Los habia vuelto a extraer hace poco, por lo que, estaban mal extraídos todos los id_player de df_match_player_miss. Esto hacia que falle la integracion de columna de jugadores en df_integrated_missing.
2. Hago assess_model_in_prod de todos los paises luego de haber perdido todos los datos por mi borrado sin querer (los que tenia los habia bajado de Drive de una copia de seguridad).
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="60">
   <si>
     <t>id_country</t>
   </si>
@@ -253,17 +253,19 @@
     <t>-0.05</t>
   </si>
   <si>
-    <t>(44, 20)</t>
+    <t>(44, 24)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy&quot;-&quot;mm&quot;-&quot;dd"/>
+    <numFmt numFmtId="165" formatCode="d/MM/yyyy"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -279,8 +281,17 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -291,6 +302,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE5CD"/>
         <bgColor rgb="FFFCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -332,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -388,6 +405,12 @@
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1073,13 +1096,13 @@
         <v>45461.0</v>
       </c>
       <c r="D8" s="15">
-        <v>148.0</v>
+        <v>386.0</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F8" s="16">
-        <v>30.0</v>
+        <v>60.0</v>
       </c>
       <c r="G8" s="7">
         <v>3.0</v>
@@ -1093,28 +1116,28 @@
       <c r="J8" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="K8" s="16"/>
+      <c r="K8" s="16">
+        <v>3.0</v>
+      </c>
       <c r="L8" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="M8" s="16" t="s">
-        <v>34</v>
-      </c>
+      <c r="M8" s="16"/>
       <c r="N8" s="17" t="s">
         <v>35</v>
       </c>
       <c r="O8" s="14">
-        <v>45463.0</v>
+        <v>45465.0</v>
       </c>
       <c r="P8" s="15" t="s">
         <v>58</v>
       </c>
       <c r="Q8" s="10">
         <f t="shared" si="3"/>
-        <v>1.351106848</v>
+        <v>1.575568182</v>
       </c>
       <c r="R8" s="18">
-        <v>1.18897402636724</v>
+        <v>1.3865</v>
       </c>
       <c r="S8" s="16">
         <v>44.0</v>
@@ -1124,9 +1147,29 @@
       </c>
       <c r="U8" s="3">
         <f t="shared" si="2"/>
-        <v>4.884770913</v>
+        <v>5.696284965</v>
       </c>
       <c r="V8" s="19"/>
+    </row>
+    <row r="11">
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="G11" s="21"/>
+    </row>
+    <row r="12">
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+    </row>
+    <row r="13">
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+    </row>
+    <row r="14">
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+    </row>
+    <row r="18">
+      <c r="I18" s="21"/>
     </row>
   </sheetData>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
Vuelvo a seleccionar mejores modelos
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="57">
   <si>
     <t>id_country</t>
   </si>
@@ -146,7 +146,7 @@
     <t>LogisticRegression</t>
   </si>
   <si>
-    <t>0.9</t>
+    <t>0.8</t>
   </si>
   <si>
     <t>0.1</t>
@@ -155,57 +155,53 @@
     <t>[1481, 1483, 1484]</t>
   </si>
   <si>
+    <t>ml</t>
+  </si>
+  <si>
+    <t>-0.2</t>
+  </si>
+  <si>
+    <t>(91, 25)</t>
+  </si>
+  <si>
+    <t>Todos los modelos de SPA tienen sesgo debido a una mala integracion. Tengo que mejorar la integracion urgentemente</t>
+  </si>
+  <si>
+    <t>italy</t>
+  </si>
+  <si>
+    <t>SVC</t>
+  </si>
+  <si>
+    <t>[771, 772, 773]</t>
+  </si>
+  <si>
+    <t>under</t>
+  </si>
+  <si>
     <t>-0.15</t>
   </si>
   <si>
-    <t>(91, 26)</t>
-  </si>
-  <si>
-    <t>Todos los modelos de SPA tienen sesgo debido a una mala integracion. Tengo que mejorar la integracion urgentemente.
-Agregue 10 partidos a los 81 que ya habia (un 12% mas)
-Cuando hace -1 y la dif_prob es muy cercana al -0.15 casi siempre voy por el 1 igual. En cambio, cuando hace -1 y la dif_prob es muy grande, voy por empate (generalmente se da el empate cuando el 1 es muy fav y mi modelo dice que no).</t>
-  </si>
-  <si>
-    <t>italy</t>
-  </si>
-  <si>
-    <t>SVC</t>
+    <t>(81, 36)</t>
+  </si>
+  <si>
+    <t>argentina</t>
   </si>
   <si>
     <t>0.2</t>
   </si>
   <si>
-    <t>[771, 772, 773]</t>
-  </si>
-  <si>
-    <t>ml</t>
-  </si>
-  <si>
-    <t>under</t>
-  </si>
-  <si>
-    <t>(80, 19)</t>
-  </si>
-  <si>
-    <t>Agregue 20 partidos a los 60 que ya habia (un 33% mas)</t>
-  </si>
-  <si>
-    <t>argentina</t>
-  </si>
-  <si>
-    <t>[61, 62, 63, 64, 65, 66, 67]</t>
-  </si>
-  <si>
-    <t>over</t>
+    <t>[61, 62, 64, 65, 66, 67]</t>
   </si>
   <si>
     <t>-0.5</t>
   </si>
   <si>
-    <t>(81, 43)</t>
-  </si>
-  <si>
-    <t>No puede predecir rdos de partidos de Riestra ni de Independiente Rivadacia (los recien ascendidos, porque no estan en el fifa 24)</t>
+    <t>(107, 25)</t>
+  </si>
+  <si>
+    <t>No puede predecir rdos de partidos de Riestra ni de Independiente Rivadacia (los recien ascendidos, porque no estan en el fifa 24)
+Es logico que ande mal porque los partidos de Copa Argentina son en estadio neutral. Sofifa no le da mucha bola a los equipos de sudamerica.</t>
   </si>
   <si>
     <t>france</t>
@@ -214,10 +210,7 @@
     <t>[551, 552, 553, 554]</t>
   </si>
   <si>
-    <t>-0.1</t>
-  </si>
-  <si>
-    <t>(47, 42)</t>
+    <t>(56, 18)</t>
   </si>
   <si>
     <t>england</t>
@@ -226,19 +219,16 @@
     <t>[481, 482, 483, 484]</t>
   </si>
   <si>
-    <t>(116, 21)</t>
+    <t>(122, 34)</t>
   </si>
   <si>
     <t>germany</t>
   </si>
   <si>
-    <t>0.8</t>
-  </si>
-  <si>
     <t>[591, 593, 594]</t>
   </si>
   <si>
-    <t>(18, 32)</t>
+    <t>(20, 32)</t>
   </si>
   <si>
     <t>usa</t>
@@ -300,8 +290,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE5CD"/>
-        <bgColor rgb="FFFCE5CD"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -349,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -360,48 +350,59 @@
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -626,6 +627,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="5" max="5" width="15.13"/>
+    <col customWidth="1" min="12" max="12" width="20.5"/>
     <col customWidth="1" min="22" max="22" width="65.13"/>
   </cols>
   <sheetData>
@@ -707,56 +709,58 @@
       <c r="C2" s="5">
         <v>45418.0</v>
       </c>
-      <c r="D2" s="3">
-        <v>365.0</v>
-      </c>
-      <c r="E2" s="6" t="s">
+      <c r="D2" s="6">
+        <v>547.0</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="6">
-        <v>30.0</v>
-      </c>
-      <c r="G2" s="6">
+      <c r="F2" s="8">
+        <v>60.0</v>
+      </c>
+      <c r="G2" s="7">
         <v>3.0</v>
       </c>
-      <c r="H2" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6" t="s">
+      <c r="H2" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="7">
-        <v>10.0</v>
-      </c>
-      <c r="L2" s="7" t="s">
+      <c r="K2" s="9"/>
+      <c r="L2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="8"/>
-      <c r="N2" s="9"/>
+      <c r="M2" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" s="4"/>
       <c r="O2" s="5">
         <v>45440.0</v>
       </c>
-      <c r="P2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q2" s="10">
-        <v>10.9504494555667</v>
-      </c>
-      <c r="R2" s="10">
-        <v>4.28944567529248</v>
-      </c>
-      <c r="S2" s="8"/>
-      <c r="T2" s="4" t="s">
+      <c r="P2" s="6" t="s">
         <v>28</v>
+      </c>
+      <c r="Q2" s="11">
+        <v>36.8495516929146</v>
+      </c>
+      <c r="R2" s="11">
+        <v>11.1750233850569</v>
+      </c>
+      <c r="S2" s="10">
+        <v>91.0</v>
+      </c>
+      <c r="T2" s="12" t="s">
+        <v>29</v>
       </c>
       <c r="U2" s="3">
         <v>40.0</v>
       </c>
-      <c r="V2" s="11" t="s">
-        <v>29</v>
+      <c r="V2" s="13" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -764,129 +768,123 @@
         <v>77.0</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="5">
         <v>45418.0</v>
       </c>
-      <c r="D3" s="3">
-        <v>520.0</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" s="7">
-        <v>60.0</v>
-      </c>
-      <c r="G3" s="7">
+      <c r="D3" s="6">
+        <v>358.0</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="10">
+        <v>30.0</v>
+      </c>
+      <c r="G3" s="9">
         <v>3.0</v>
       </c>
-      <c r="H3" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="8"/>
-      <c r="J3" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" s="7">
-        <v>10.0</v>
-      </c>
-      <c r="L3" s="7" t="s">
+      <c r="H3" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="9"/>
+      <c r="N3" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="O3" s="14">
+        <v>45465.0</v>
+      </c>
+      <c r="P3" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="O3" s="5">
-        <v>45440.0</v>
-      </c>
-      <c r="P3" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="Q3" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="R3" s="10">
-        <v>0.624947833518396</v>
-      </c>
-      <c r="S3" s="8"/>
-      <c r="T3" s="4" t="s">
+      <c r="Q3" s="11">
+        <v>0.0598</v>
+      </c>
+      <c r="R3" s="11">
+        <v>0.747445629288458</v>
+      </c>
+      <c r="S3" s="10">
+        <v>81.0</v>
+      </c>
+      <c r="T3" s="12" t="s">
         <v>36</v>
       </c>
       <c r="U3" s="3">
         <f t="shared" ref="U3:U4" si="1">Q3*$U$5/$Q$5</f>
-        <v>5.423076923</v>
-      </c>
-      <c r="V3" s="12" t="s">
-        <v>37</v>
-      </c>
+        <v>0.1587425949</v>
+      </c>
+      <c r="V3" s="15"/>
     </row>
     <row r="4">
       <c r="A4" s="3">
         <v>6.0</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" s="5">
         <v>45419.0</v>
       </c>
-      <c r="D4" s="3">
-        <v>1062.0</v>
-      </c>
-      <c r="E4" s="7" t="s">
+      <c r="D4" s="6">
+        <v>631.0</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="9">
         <v>30.0</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="9">
         <v>3.0</v>
       </c>
-      <c r="H4" s="7" t="b">
+      <c r="H4" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="7">
-        <v>10.0</v>
-      </c>
-      <c r="L4" s="7" t="s">
+      <c r="I4" s="9"/>
+      <c r="J4" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="10">
+        <v>3.0</v>
+      </c>
+      <c r="L4" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="M4" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="N4" s="4" t="s">
+      <c r="M4" s="9"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="14">
+        <v>45465.0</v>
+      </c>
+      <c r="P4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="O4" s="5">
-        <v>45440.0</v>
-      </c>
-      <c r="P4" s="3" t="s">
+      <c r="Q4" s="16">
+        <v>0.0148224109336046</v>
+      </c>
+      <c r="R4" s="11">
+        <v>0.152</v>
+      </c>
+      <c r="S4" s="10">
+        <v>107.0</v>
+      </c>
+      <c r="T4" s="12" t="s">
         <v>41</v>
-      </c>
-      <c r="Q4" s="10">
-        <v>0.0953658225050433</v>
-      </c>
-      <c r="R4" s="10">
-        <v>0.3307</v>
-      </c>
-      <c r="S4" s="8"/>
-      <c r="T4" s="4" t="s">
-        <v>42</v>
       </c>
       <c r="U4" s="3">
         <f t="shared" si="1"/>
-        <v>0.3447841275</v>
-      </c>
-      <c r="V4" s="12" t="s">
-        <v>43</v>
+        <v>0.03934695608</v>
+      </c>
+      <c r="V4" s="17" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="5">
@@ -894,135 +892,134 @@
         <v>55.0</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="5">
         <v>45419.0</v>
       </c>
-      <c r="D5" s="3">
-        <v>1348.0</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="7">
-        <v>60.0</v>
-      </c>
-      <c r="G5" s="7">
+      <c r="D5" s="6">
+        <v>91.0</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="10">
+        <v>30.0</v>
+      </c>
+      <c r="G5" s="9">
         <v>3.0</v>
       </c>
-      <c r="H5" s="7" t="b">
+      <c r="H5" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="7">
-        <v>10.0</v>
-      </c>
-      <c r="L5" s="7" t="s">
+      <c r="J5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="K5" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="M5" s="9"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="14">
+        <v>45465.0</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q5" s="11">
+        <v>15.0684194244387</v>
+      </c>
+      <c r="R5" s="11">
+        <v>7.94996514671098</v>
+      </c>
+      <c r="S5" s="10">
+        <v>56.0</v>
+      </c>
+      <c r="T5" s="12" t="s">
         <v>45</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="N5" s="9"/>
-      <c r="O5" s="5">
-        <v>45431.0</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q5" s="13">
-        <f>50*R5/47</f>
-        <v>11.06382979</v>
-      </c>
-      <c r="R5" s="10">
-        <v>10.4</v>
-      </c>
-      <c r="S5" s="7">
-        <v>52.0</v>
-      </c>
-      <c r="T5" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="U5" s="3">
         <v>40.0</v>
       </c>
-      <c r="V5" s="8"/>
+      <c r="V5" s="18"/>
     </row>
     <row r="6">
       <c r="A6" s="3">
         <v>48.0</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C6" s="5">
         <v>45419.0</v>
       </c>
-      <c r="D6" s="3">
-        <v>74.0</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="7">
-        <v>30.0</v>
-      </c>
-      <c r="G6" s="7">
+      <c r="D6" s="6">
+        <v>808.0</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="10">
+        <v>60.0</v>
+      </c>
+      <c r="G6" s="9">
         <v>3.0</v>
       </c>
-      <c r="H6" s="7" t="b">
+      <c r="H6" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="I6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="K6" s="7">
-        <v>5.0</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="M6" s="8"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="10">
+        <v>3.0</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="N6" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="O6" s="5">
-        <v>45431.0</v>
+        <v>34</v>
+      </c>
+      <c r="O6" s="14">
+        <v>45465.0</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q6" s="10">
-        <v>0.0815</v>
-      </c>
-      <c r="R6" s="10">
-        <v>0.5371</v>
-      </c>
-      <c r="S6" s="7">
+        <v>40</v>
+      </c>
+      <c r="Q6" s="11">
+        <v>0.52</v>
+      </c>
+      <c r="R6" s="11">
+        <v>4.31413684333713</v>
+      </c>
+      <c r="S6" s="9">
         <v>122.0</v>
       </c>
-      <c r="T6" s="4" t="s">
-        <v>50</v>
+      <c r="T6" s="12" t="s">
+        <v>48</v>
       </c>
       <c r="U6" s="3">
         <f t="shared" ref="U6:U8" si="2">Q6*$U$5/$Q$5</f>
-        <v>0.2946538462</v>
-      </c>
-      <c r="V6" s="8"/>
+        <v>1.38037039</v>
+      </c>
+      <c r="V6" s="18"/>
     </row>
     <row r="7">
       <c r="A7" s="3">
         <v>59.0</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C7" s="5">
         <v>45421.0</v>
@@ -1030,148 +1027,165 @@
       <c r="D7" s="3">
         <v>1757.0</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="7">
+      <c r="E7" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="9">
         <v>60.0</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="9">
         <v>3.0</v>
       </c>
-      <c r="H7" s="7" t="b">
+      <c r="H7" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="J7" s="7" t="s">
+      <c r="I7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="9">
         <v>3.0</v>
       </c>
-      <c r="L7" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="M7" s="7" t="s">
+      <c r="L7" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="N7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="O7" s="5">
-        <v>45431.0</v>
+      <c r="O7" s="14">
+        <v>45465.0</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q7" s="13">
-        <f t="shared" ref="Q7:Q8" si="3">50*R7/S7</f>
-        <v>0.6944444444</v>
-      </c>
-      <c r="R7" s="10">
-        <v>0.25</v>
-      </c>
-      <c r="S7" s="7">
-        <v>18.0</v>
-      </c>
-      <c r="T7" s="4" t="s">
-        <v>54</v>
+        <v>40</v>
+      </c>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="11">
+        <v>0.2</v>
+      </c>
+      <c r="S7" s="10">
+        <v>20.0</v>
+      </c>
+      <c r="T7" s="12" t="s">
+        <v>51</v>
       </c>
       <c r="U7" s="3">
         <f t="shared" si="2"/>
-        <v>2.510683761</v>
-      </c>
-      <c r="V7" s="8"/>
+        <v>0</v>
+      </c>
+      <c r="V7" s="18"/>
     </row>
     <row r="8">
-      <c r="A8" s="3">
+      <c r="A8" s="20">
         <v>167.0</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>55</v>
+      <c r="B8" s="21" t="s">
+        <v>52</v>
       </c>
       <c r="C8" s="14">
         <v>45461.0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="6">
         <v>386.0</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="10">
         <v>60.0</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="9">
         <v>3.0</v>
       </c>
-      <c r="H8" s="16" t="b">
+      <c r="H8" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="I8" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="J8" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="K8" s="16">
+      <c r="I8" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="K8" s="10">
         <v>3.0</v>
       </c>
-      <c r="L8" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="M8" s="16"/>
-      <c r="N8" s="17" t="s">
-        <v>35</v>
+      <c r="L8" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="M8" s="10"/>
+      <c r="N8" s="12" t="s">
+        <v>34</v>
       </c>
       <c r="O8" s="14">
         <v>45465.0</v>
       </c>
-      <c r="P8" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q8" s="10">
-        <f t="shared" si="3"/>
+      <c r="P8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q8" s="19">
+        <f>50*R8/S8</f>
         <v>1.575568182</v>
       </c>
-      <c r="R8" s="18">
+      <c r="R8" s="11">
         <v>1.3865</v>
       </c>
-      <c r="S8" s="16">
+      <c r="S8" s="10">
         <v>44.0</v>
       </c>
-      <c r="T8" s="17" t="s">
-        <v>59</v>
+      <c r="T8" s="12" t="s">
+        <v>56</v>
       </c>
       <c r="U8" s="3">
         <f t="shared" si="2"/>
-        <v>5.696284965</v>
-      </c>
-      <c r="V8" s="19"/>
+        <v>4.182437819</v>
+      </c>
+      <c r="V8" s="22"/>
     </row>
     <row r="11">
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="G11" s="21"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="G11" s="24"/>
     </row>
     <row r="12">
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
     </row>
     <row r="13">
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
     </row>
     <row r="14">
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
     </row>
     <row r="18">
-      <c r="I18" s="21"/>
+      <c r="I18" s="24"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="S2:S8">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FFFFD666"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R8">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FF57BB8A"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Recollect df_match_player and train models for USA
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="55">
   <si>
     <t>id_country</t>
   </si>
@@ -234,16 +234,10 @@
     <t>usa</t>
   </si>
   <si>
-    <t>0.7</t>
-  </si>
-  <si>
     <t>[1671, 1672]</t>
   </si>
   <si>
-    <t>-0.05</t>
-  </si>
-  <si>
-    <t>(44, 24)</t>
+    <t>(58, 45)</t>
   </si>
 </sst>
 </file>
@@ -281,18 +275,12 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -339,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -398,19 +386,13 @@
     <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -1080,17 +1062,17 @@
       <c r="V7" s="18"/>
     </row>
     <row r="8">
-      <c r="A8" s="20">
+      <c r="A8" s="3">
         <v>167.0</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="4" t="s">
         <v>52</v>
       </c>
       <c r="C8" s="14">
-        <v>45461.0</v>
+        <v>45467.0</v>
       </c>
       <c r="D8" s="6">
-        <v>386.0</v>
+        <v>668.0</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>23</v>
@@ -1102,68 +1084,68 @@
         <v>3.0</v>
       </c>
       <c r="H8" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="L8" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="J8" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="K8" s="10">
-        <v>3.0</v>
-      </c>
-      <c r="L8" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="M8" s="10"/>
+      <c r="M8" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="N8" s="12" t="s">
         <v>34</v>
       </c>
       <c r="O8" s="14">
-        <v>45465.0</v>
-      </c>
-      <c r="P8" s="6" t="s">
-        <v>55</v>
+        <v>45467.0</v>
+      </c>
+      <c r="P8" s="6">
+        <v>0.0</v>
       </c>
       <c r="Q8" s="19">
         <f>50*R8/S8</f>
-        <v>1.575568182</v>
+        <v>0.148362069</v>
       </c>
       <c r="R8" s="11">
-        <v>1.3865</v>
+        <v>0.1721</v>
       </c>
       <c r="S8" s="10">
-        <v>44.0</v>
+        <v>58.0</v>
       </c>
       <c r="T8" s="12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="U8" s="3">
         <f t="shared" si="2"/>
-        <v>4.182437819</v>
-      </c>
-      <c r="V8" s="22"/>
+        <v>0.3938357827</v>
+      </c>
+      <c r="V8" s="20"/>
     </row>
     <row r="11">
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="G11" s="24"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="G11" s="22"/>
     </row>
     <row r="12">
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13">
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
     </row>
     <row r="14">
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
     </row>
     <row r="18">
-      <c r="I18" s="24"/>
+      <c r="I18" s="22"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="S2:S8">

</xml_diff>

<commit_message>
Selecciono nuevo mejor modelo usa y automatizo el m para variar el stake
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="56">
   <si>
     <t>id_country</t>
   </si>
@@ -237,7 +237,17 @@
     <t>[1671, 1672]</t>
   </si>
   <si>
-    <t>(58, 45)</t>
+    <t>(58, 15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parece que es poco 17% pero si pongo los 700k en 4 fechas, tendria cerca de 69 Millones (es decir, 69000 dolares). 
+Criterio:
+- bal_type = under
+- n_years_to_select &gt;= 10 --&gt; estabilidad al modelo
+- thr_prob_min_best = -0.5 --&gt; no esta overfitteado, la prediccion del modelo es lo que apostas.
+- Variables seleccionadas son solo 15 pero tienen sentido.
+- Me cierran las predicciones
+</t>
   </si>
 </sst>
 </file>
@@ -1072,7 +1082,7 @@
         <v>45467.0</v>
       </c>
       <c r="D8" s="6">
-        <v>668.0</v>
+        <v>544.0</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>23</v>
@@ -1084,11 +1094,13 @@
         <v>3.0</v>
       </c>
       <c r="H8" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="I8" s="10"/>
+        <v>1</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>24</v>
+      </c>
       <c r="J8" s="10" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="K8" s="10">
         <v>5.0</v>
@@ -1105,15 +1117,14 @@
       <c r="O8" s="14">
         <v>45467.0</v>
       </c>
-      <c r="P8" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="Q8" s="19">
-        <f>50*R8/S8</f>
-        <v>0.148362069</v>
+      <c r="P8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q8" s="11">
+        <v>0.1293</v>
       </c>
       <c r="R8" s="11">
-        <v>0.1721</v>
+        <v>0.1172</v>
       </c>
       <c r="S8" s="10">
         <v>58.0</v>
@@ -1123,14 +1134,20 @@
       </c>
       <c r="U8" s="3">
         <f t="shared" si="2"/>
-        <v>0.3938357827</v>
-      </c>
-      <c r="V8" s="20"/>
+        <v>0.3432344066</v>
+      </c>
+      <c r="V8" s="20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="G10" s="22"/>
     </row>
     <row r="11">
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
-      <c r="G11" s="22"/>
     </row>
     <row r="12">
       <c r="C12" s="21"/>
@@ -1140,12 +1157,8 @@
       <c r="C13" s="21"/>
       <c r="D13" s="21"/>
     </row>
-    <row r="14">
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-    </row>
-    <row r="18">
-      <c r="I18" s="22"/>
+    <row r="17">
+      <c r="I17" s="22"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="S2:S8">

</xml_diff>

<commit_message>
Arreglo error en mnm.py y vuelvo a seleccionar mejor modelo para USA
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="56">
   <si>
     <t>id_country</t>
   </si>
@@ -234,20 +234,13 @@
     <t>usa</t>
   </si>
   <si>
+    <t>0.9</t>
+  </si>
+  <si>
     <t>[1671, 1672]</t>
   </si>
   <si>
-    <t>(58, 15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parece que es poco 17% pero si pongo los 700k en 4 fechas, tendria cerca de 69 Millones (es decir, 69000 dolares). 
-Criterio:
-- bal_type = under
-- n_years_to_select &gt;= 10 --&gt; estabilidad al modelo
-- thr_prob_min_best = -0.5 --&gt; no esta overfitteado, la prediccion del modelo es lo que apostas.
-- Variables seleccionadas son solo 15 pero tienen sentido.
-- Me cierran las predicciones
-</t>
+    <t>(72, 30)</t>
   </si>
 </sst>
 </file>
@@ -1082,63 +1075,59 @@
         <v>45467.0</v>
       </c>
       <c r="D8" s="6">
-        <v>544.0</v>
+        <v>219.0</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>23</v>
       </c>
       <c r="F8" s="10">
-        <v>60.0</v>
+        <v>30.0</v>
       </c>
       <c r="G8" s="9">
         <v>3.0</v>
       </c>
       <c r="H8" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K8" s="10">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N8" s="12" t="s">
-        <v>34</v>
-      </c>
+      <c r="N8" s="12"/>
       <c r="O8" s="14">
-        <v>45467.0</v>
+        <v>45473.0</v>
       </c>
       <c r="P8" s="6" t="s">
         <v>40</v>
       </c>
       <c r="Q8" s="11">
-        <v>0.1293</v>
+        <v>0.0111</v>
       </c>
       <c r="R8" s="11">
-        <v>0.1172</v>
+        <v>1.98</v>
       </c>
       <c r="S8" s="10">
-        <v>58.0</v>
+        <v>72.0</v>
       </c>
       <c r="T8" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="U8" s="3">
         <f t="shared" si="2"/>
-        <v>0.3432344066</v>
-      </c>
-      <c r="V8" s="20" t="s">
-        <v>55</v>
-      </c>
+        <v>0.02946559871</v>
+      </c>
+      <c r="V8" s="20"/>
     </row>
     <row r="10">
       <c r="C10" s="21"/>

</xml_diff>

<commit_message>
Nuevo assess argentina y seleccion de modelo
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="57">
   <si>
     <t>id_country</t>
   </si>
@@ -222,8 +222,96 @@
     <t>[61, 62, 64, 65, 66, 67]</t>
   </si>
   <si>
-    <t>No puede predecir rdos de partidos de Riestra ni de Independiente Rivadacia (los recien ascendidos, porque no estan en el fifa 24)
-Es logico que ande mal porque los partidos de Copa Argentina son en estadio neutral. Sofifa no le da mucha bola a los equipos de sudamerica.</t>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">- No puede predecir rdos de partidos de Riestra ni de Independiente Rivadavia (los recien ascendidos, porque no estan en el fifa 24)
+- Es logico que ande mal porque los partidos de Copa Argentina son en estadio neutral. Sofifa no le da mucha bola a los equipos de sudamerica.
+Si bien no es el que mas roi_pp tiene, es el primero con under y n_years_to_select &gt;= 10.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>n_years            Average of roi_por_partido</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+3   </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">     </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">             </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t>0,06</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">5                       0,01
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>10                     0,17
+None                 0,14</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Grand Total       0,09</t>
+    </r>
   </si>
   <si>
     <t>x</t>
@@ -1185,7 +1273,7 @@
         <v>45419.0</v>
       </c>
       <c r="D8" s="9">
-        <v>631.0</v>
+        <v>779.0</v>
       </c>
       <c r="E8" s="12">
         <v>30.0</v>
@@ -1201,45 +1289,49 @@
         <v>35</v>
       </c>
       <c r="J8" s="13">
-        <v>3.0</v>
+        <v>10.0</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
+      <c r="L8" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="M8" s="12" t="s">
+        <v>42</v>
+      </c>
       <c r="N8" s="20" t="s">
         <v>30</v>
       </c>
       <c r="O8" s="15">
-        <v>25.0</v>
+        <v>21.0</v>
       </c>
       <c r="P8" s="21">
-        <v>45465.0</v>
+        <v>45488.0</v>
       </c>
       <c r="Q8" s="6" t="s">
         <v>43</v>
       </c>
       <c r="R8" s="29">
-        <v>0.0148224109336046</v>
+        <v>-6.0E-4</v>
       </c>
       <c r="S8" s="16">
-        <v>16.264</v>
+        <v>8.39</v>
       </c>
       <c r="T8" s="13">
-        <v>107.0</v>
+        <v>92.0</v>
       </c>
       <c r="U8" s="16">
         <f t="shared" si="1"/>
-        <v>0.152</v>
+        <v>0.09119565217</v>
       </c>
       <c r="V8" s="16">
         <f t="shared" si="2"/>
-        <v>0.0228</v>
+        <v>0.01367934783</v>
       </c>
       <c r="W8" s="6">
         <f t="shared" si="3"/>
-        <v>0.4080528374</v>
+        <v>0.2448200304</v>
       </c>
       <c r="X8" s="30" t="s">
         <v>54</v>

</xml_diff>

<commit_message>
Nuevo assess de USA
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Hoja 1" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Hoja 2" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Hoja 1'!$A$1:$X$8</definedName>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="55">
   <si>
     <t>id_country</t>
   </si>
@@ -132,9 +133,6 @@
     <t>Observaciones</t>
   </si>
   <si>
-    <t>Parametros para apostar</t>
-  </si>
-  <si>
     <t>spain</t>
   </si>
   <si>
@@ -159,9 +157,6 @@
     <t>Todos los modelos de SPA tienen sesgo debido a una mala integracion. Tengo que mejorar la integracion urgentemente</t>
   </si>
   <si>
-    <t>ROI asses --&gt; ROI realidad</t>
-  </si>
-  <si>
     <t>france</t>
   </si>
   <si>
@@ -177,9 +172,6 @@
     <t>-0.15</t>
   </si>
   <si>
-    <t>max m</t>
-  </si>
-  <si>
     <t>england</t>
   </si>
   <si>
@@ -190,9 +182,6 @@
   </si>
   <si>
     <t>-0.5</t>
-  </si>
-  <si>
-    <t>max roi pp</t>
   </si>
   <si>
     <t>usa</t>
@@ -310,14 +299,37 @@
         <color theme="1"/>
       </rPr>
       <t xml:space="preserve">
-Grand Total       0,09</t>
+Grand Total       0,09
+</t>
     </r>
-  </si>
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>y</t>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>No apostaria en ARG:</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Todos los modelos de ARG son bastante pedorros. Solo 800 modelos de 2300, tienen rentabilidad al menos 0 o mas de rentabilidad. Ademas, se juega todos los dias y para un apostador te mata. </t>
+    </r>
+  </si>
+  <si>
+    <t>Parametros para apostar</t>
+  </si>
+  <si>
+    <t>ROI asses --&gt; ROI realidad</t>
+  </si>
+  <si>
+    <t>max m</t>
+  </si>
+  <si>
+    <t>max roi pp</t>
   </si>
 </sst>
 </file>
@@ -342,12 +354,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -359,6 +365,12 @@
     <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -429,87 +441,87 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="9" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="9" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -519,6 +531,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -801,568 +817,536 @@
       <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="5" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="5">
+        <v>148.0</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6">
-        <v>148.0</v>
-      </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7">
+        <v>45418.0</v>
+      </c>
+      <c r="D2" s="8">
+        <v>547.0</v>
+      </c>
+      <c r="E2" s="9">
+        <v>60.0</v>
+      </c>
+      <c r="F2" s="10">
+        <v>3.0</v>
+      </c>
+      <c r="G2" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="8">
-        <v>45418.0</v>
-      </c>
-      <c r="D2" s="9">
-        <v>547.0</v>
-      </c>
-      <c r="E2" s="10">
-        <v>60.0</v>
-      </c>
-      <c r="F2" s="11">
-        <v>3.0</v>
-      </c>
-      <c r="G2" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="10" t="s">
+      <c r="I2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="J2" s="11"/>
+      <c r="K2" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12" t="s">
+      <c r="L2" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="M2" s="11"/>
+      <c r="N2" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="M2" s="12"/>
-      <c r="N2" s="14" t="s">
+      <c r="O2" s="14">
+        <v>25.0</v>
+      </c>
+      <c r="P2" s="7">
+        <v>45440.0</v>
+      </c>
+      <c r="Q2" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="O2" s="15">
-        <v>25.0</v>
-      </c>
-      <c r="P2" s="8">
-        <v>45440.0</v>
-      </c>
-      <c r="Q2" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="R2" s="16">
+      <c r="R2" s="15">
         <v>36.8495516929146</v>
       </c>
-      <c r="S2" s="16">
+      <c r="S2" s="15">
         <v>1016.9271280401779</v>
       </c>
-      <c r="T2" s="13">
+      <c r="T2" s="12">
         <v>91.0</v>
       </c>
-      <c r="U2" s="16">
+      <c r="U2" s="15">
         <f t="shared" ref="U2:U8" si="1">S2/T2</f>
         <v>11.17502339</v>
       </c>
-      <c r="V2" s="16">
-        <f t="shared" ref="V2:V8" si="2">$AA$2*U2</f>
+      <c r="V2" s="15">
+        <f>'Hoja 2'!$B$2*U2</f>
         <v>1.676253508</v>
       </c>
-      <c r="W2" s="6">
-        <f t="shared" ref="W2:W8" si="3">U2*$AA$3/$AA$4</f>
+      <c r="W2" s="5">
+        <f>U2*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
         <v>30</v>
       </c>
-      <c r="X2" s="17" t="s">
+      <c r="X2" s="16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5">
+        <v>55.0</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="Z2" s="18" t="s">
+      <c r="C3" s="7">
+        <v>45419.0</v>
+      </c>
+      <c r="D3" s="8">
+        <v>91.0</v>
+      </c>
+      <c r="E3" s="12">
+        <v>30.0</v>
+      </c>
+      <c r="F3" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="AA2" s="19">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6">
-        <v>55.0</v>
-      </c>
-      <c r="B3" s="7" t="s">
+      <c r="J3" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="K3" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="8">
-        <v>45419.0</v>
-      </c>
-      <c r="D3" s="9">
-        <v>91.0</v>
-      </c>
-      <c r="E3" s="13">
-        <v>30.0</v>
-      </c>
-      <c r="F3" s="12">
-        <v>3.0</v>
-      </c>
-      <c r="G3" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="13" t="s">
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="J3" s="13">
-        <v>5.0</v>
-      </c>
-      <c r="K3" s="12" t="s">
+      <c r="O3" s="14">
+        <v>18.0</v>
+      </c>
+      <c r="P3" s="18">
+        <v>45465.0</v>
+      </c>
+      <c r="Q3" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="O3" s="15">
-        <v>18.0</v>
-      </c>
-      <c r="P3" s="21">
-        <v>45465.0</v>
-      </c>
-      <c r="Q3" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="R3" s="16">
+      <c r="R3" s="15">
         <v>15.0684194244387</v>
       </c>
-      <c r="S3" s="16">
+      <c r="S3" s="15">
         <v>445.1980482158149</v>
       </c>
-      <c r="T3" s="13">
+      <c r="T3" s="12">
         <v>56.0</v>
       </c>
-      <c r="U3" s="16">
+      <c r="U3" s="15">
         <f t="shared" si="1"/>
         <v>7.949965147</v>
       </c>
-      <c r="V3" s="16">
-        <f t="shared" si="2"/>
+      <c r="V3" s="15">
+        <f>'Hoja 2'!$B$2*U3</f>
         <v>1.192494772</v>
       </c>
-      <c r="W3" s="6">
-        <f t="shared" si="3"/>
+      <c r="W3" s="5">
+        <f>U3*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
         <v>21.34214365</v>
       </c>
-      <c r="X3" s="22"/>
-      <c r="Z3" s="5" t="s">
+      <c r="X3" s="19"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5">
+        <v>48.0</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="7">
+        <v>45419.0</v>
+      </c>
+      <c r="D4" s="8">
+        <v>808.0</v>
+      </c>
+      <c r="E4" s="12">
+        <v>60.0</v>
+      </c>
+      <c r="F4" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G4" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="M4" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="AA3" s="18">
-        <v>30.0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6">
-        <v>48.0</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="N4" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="O4" s="14">
+        <v>34.0</v>
+      </c>
+      <c r="P4" s="18">
+        <v>45465.0</v>
+      </c>
+      <c r="Q4" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="8">
-        <v>45419.0</v>
-      </c>
-      <c r="D4" s="9">
-        <v>808.0</v>
-      </c>
-      <c r="E4" s="13">
-        <v>60.0</v>
-      </c>
-      <c r="F4" s="12">
-        <v>3.0</v>
-      </c>
-      <c r="G4" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="J4" s="13">
-        <v>3.0</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="L4" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="M4" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="N4" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="O4" s="15">
-        <v>34.0</v>
-      </c>
-      <c r="P4" s="21">
-        <v>45465.0</v>
-      </c>
-      <c r="Q4" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="R4" s="16">
+      <c r="R4" s="15">
         <v>0.52</v>
       </c>
-      <c r="S4" s="16">
+      <c r="S4" s="15">
         <v>526.3246948871299</v>
       </c>
-      <c r="T4" s="12">
+      <c r="T4" s="11">
         <v>122.0</v>
       </c>
-      <c r="U4" s="16">
+      <c r="U4" s="15">
         <f t="shared" si="1"/>
         <v>4.314136843</v>
       </c>
-      <c r="V4" s="16">
-        <f t="shared" si="2"/>
+      <c r="V4" s="15">
+        <f>'Hoja 2'!$B$2*U4</f>
         <v>0.6471205265</v>
       </c>
-      <c r="W4" s="6">
-        <f t="shared" si="3"/>
+      <c r="W4" s="5">
+        <f>U4*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
         <v>11.58155118</v>
       </c>
-      <c r="X4" s="22"/>
-      <c r="Z4" s="5" t="s">
+      <c r="X4" s="19"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5">
+        <v>167.0</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="18">
+        <v>45467.0</v>
+      </c>
+      <c r="D5" s="8">
+        <v>219.0</v>
+      </c>
+      <c r="E5" s="12">
+        <v>30.0</v>
+      </c>
+      <c r="F5" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G5" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="M5" s="12"/>
+      <c r="N5" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" s="14">
+        <v>30.0</v>
+      </c>
+      <c r="P5" s="18">
+        <v>45491.0</v>
+      </c>
+      <c r="Q5" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="R5" s="15">
+        <v>0.066468</v>
+      </c>
+      <c r="S5" s="15">
+        <v>355.07</v>
+      </c>
+      <c r="T5" s="12">
+        <v>125.0</v>
+      </c>
+      <c r="U5" s="15">
+        <f t="shared" si="1"/>
+        <v>2.84056</v>
+      </c>
+      <c r="V5" s="15">
+        <f>'Hoja 2'!$B$2*U5</f>
+        <v>0.426084</v>
+      </c>
+      <c r="W5" s="5">
+        <f>U5*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
+        <v>7.625648472</v>
+      </c>
+      <c r="X5" s="21"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5">
+        <v>77.0</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="AA4" s="24">
-        <f>MAX(U2:U8)</f>
-        <v>11.17502339</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6">
-        <v>167.0</v>
-      </c>
-      <c r="B5" s="7" t="s">
+      <c r="C6" s="7">
+        <v>45418.0</v>
+      </c>
+      <c r="D6" s="8">
+        <v>358.0</v>
+      </c>
+      <c r="E6" s="12">
+        <v>30.0</v>
+      </c>
+      <c r="F6" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G6" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="21">
-        <v>45467.0</v>
-      </c>
-      <c r="D5" s="9">
-        <v>219.0</v>
-      </c>
-      <c r="E5" s="13">
-        <v>30.0</v>
-      </c>
-      <c r="F5" s="12">
-        <v>3.0</v>
-      </c>
-      <c r="G5" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="I5" s="13" t="s">
+      <c r="L6" s="11"/>
+      <c r="M6" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="13">
-        <v>3.0</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="L5" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="M5" s="13"/>
-      <c r="N5" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="O5" s="15">
-        <v>30.0</v>
-      </c>
-      <c r="P5" s="21">
-        <v>45487.0</v>
-      </c>
-      <c r="Q5" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="R5" s="16">
-        <v>0.066468</v>
-      </c>
-      <c r="S5" s="16">
-        <v>196.45</v>
-      </c>
-      <c r="T5" s="13">
-        <v>111.0</v>
-      </c>
-      <c r="U5" s="16">
-        <f t="shared" si="1"/>
-        <v>1.76981982</v>
-      </c>
-      <c r="V5" s="16">
-        <f t="shared" si="2"/>
-        <v>0.265472973</v>
-      </c>
-      <c r="W5" s="6">
-        <f t="shared" si="3"/>
-        <v>4.751184205</v>
-      </c>
-      <c r="X5" s="25"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6">
-        <v>77.0</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" s="8">
-        <v>45418.0</v>
-      </c>
-      <c r="D6" s="9">
-        <v>358.0</v>
-      </c>
-      <c r="E6" s="13">
-        <v>30.0</v>
-      </c>
-      <c r="F6" s="12">
-        <v>3.0</v>
-      </c>
-      <c r="G6" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="N6" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="O6" s="15">
+      <c r="O6" s="14">
         <v>36.0</v>
       </c>
-      <c r="P6" s="21">
+      <c r="P6" s="18">
         <v>45465.0</v>
       </c>
-      <c r="Q6" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="R6" s="16">
+      <c r="Q6" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="R6" s="15">
         <v>0.0598</v>
       </c>
-      <c r="S6" s="16">
+      <c r="S6" s="15">
         <v>60.5430959723651</v>
       </c>
-      <c r="T6" s="13">
+      <c r="T6" s="12">
         <v>81.0</v>
       </c>
-      <c r="U6" s="16">
+      <c r="U6" s="15">
         <f t="shared" si="1"/>
         <v>0.7474456293</v>
       </c>
-      <c r="V6" s="16">
-        <f t="shared" si="2"/>
+      <c r="V6" s="15">
+        <f>'Hoja 2'!$B$2*U6</f>
         <v>0.1121168444</v>
       </c>
-      <c r="W6" s="6">
-        <f t="shared" si="3"/>
+      <c r="W6" s="5">
+        <f>U6*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
         <v>2.006561249</v>
       </c>
-      <c r="X6" s="26"/>
+      <c r="X6" s="22"/>
     </row>
     <row r="7">
-      <c r="A7" s="6">
+      <c r="A7" s="5">
         <v>59.0</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" s="8">
+      <c r="B7" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="7">
         <v>45421.0</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <v>1757.0</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="11">
         <v>60.0</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="11">
         <v>3.0</v>
       </c>
-      <c r="G7" s="12" t="b">
+      <c r="G7" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="12">
+      <c r="J7" s="11">
         <v>3.0</v>
       </c>
-      <c r="K7" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="L7" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="M7" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="N7" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="O7" s="15">
+      <c r="K7" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="O7" s="14">
         <v>32.0</v>
       </c>
-      <c r="P7" s="21">
+      <c r="P7" s="18">
         <v>45465.0</v>
       </c>
-      <c r="Q7" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="R7" s="27"/>
-      <c r="S7" s="16">
+      <c r="Q7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="R7" s="23"/>
+      <c r="S7" s="15">
         <v>4.0</v>
       </c>
-      <c r="T7" s="13">
+      <c r="T7" s="12">
         <v>20.0</v>
       </c>
-      <c r="U7" s="16">
+      <c r="U7" s="15">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="V7" s="16">
-        <f t="shared" si="2"/>
+      <c r="V7" s="15">
+        <f>'Hoja 2'!$B$2*U7</f>
         <v>0.03</v>
       </c>
-      <c r="W7" s="6">
-        <f t="shared" si="3"/>
+      <c r="W7" s="5">
+        <f>U7*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
         <v>0.5369116281</v>
       </c>
-      <c r="X7" s="22"/>
-      <c r="Z7" s="28">
+      <c r="X7" s="19"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5">
+        <v>6.0</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="7">
+        <v>45419.0</v>
+      </c>
+      <c r="D8" s="8">
+        <v>779.0</v>
+      </c>
+      <c r="E8" s="11">
         <v>30.0</v>
       </c>
-      <c r="AA7" s="28">
-        <v>1118.0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6">
-        <v>6.0</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="8">
-        <v>45419.0</v>
-      </c>
-      <c r="D8" s="9">
-        <v>779.0</v>
-      </c>
-      <c r="E8" s="12">
-        <v>30.0</v>
-      </c>
-      <c r="F8" s="12">
+      <c r="F8" s="11">
         <v>3.0</v>
       </c>
-      <c r="G8" s="12" t="b">
+      <c r="G8" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="12"/>
-      <c r="I8" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" s="13">
+      <c r="H8" s="11"/>
+      <c r="I8" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="J8" s="12">
         <v>10.0</v>
       </c>
-      <c r="K8" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="L8" s="12" t="s">
+      <c r="K8" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="N8" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="M8" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="N8" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="O8" s="15">
+      <c r="O8" s="14">
         <v>21.0</v>
       </c>
-      <c r="P8" s="21">
+      <c r="P8" s="18">
         <v>45488.0</v>
       </c>
-      <c r="Q8" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="R8" s="29">
+      <c r="Q8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="R8" s="24">
         <v>-6.0E-4</v>
       </c>
-      <c r="S8" s="16">
+      <c r="S8" s="15">
         <v>8.39</v>
       </c>
-      <c r="T8" s="13">
+      <c r="T8" s="12">
         <v>92.0</v>
       </c>
-      <c r="U8" s="16">
+      <c r="U8" s="15">
         <f t="shared" si="1"/>
         <v>0.09119565217</v>
       </c>
-      <c r="V8" s="16">
-        <f t="shared" si="2"/>
+      <c r="V8" s="15">
+        <f>'Hoja 2'!$B$2*U8</f>
         <v>0.01367934783</v>
       </c>
-      <c r="W8" s="6">
-        <f t="shared" si="3"/>
+      <c r="W8" s="5">
+        <f>U8*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
         <v>0.2448200304</v>
       </c>
-      <c r="X8" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="Z8" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="AA8" s="28" t="s">
-        <v>56</v>
-      </c>
+      <c r="X8" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z8" s="26"/>
+      <c r="AA8" s="26"/>
     </row>
     <row r="10">
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="F10" s="32"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="F10" s="28"/>
     </row>
     <row r="11">
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="W11" s="33"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="W11" s="29"/>
     </row>
     <row r="12">
-      <c r="C12" s="31"/>
-      <c r="D12" s="31"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
     </row>
     <row r="13">
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
     </row>
     <row r="17">
-      <c r="H17" s="32"/>
+      <c r="H17" s="28"/>
     </row>
   </sheetData>
   <autoFilter ref="$A$1:$X$8">
@@ -1403,4 +1387,54 @@
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="32">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="31">
+        <v>30.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="33">
+        <f>MAX('Hoja 1'!U2:U8)</f>
+        <v>11.17502339</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26">
+        <v>30.0</v>
+      </c>
+      <c r="B7" s="26">
+        <v>1118.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Nuevo assess model USA y cambio de modelo
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -184,6 +184,12 @@
     <t>-0.5</t>
   </si>
   <si>
+    <t>italy</t>
+  </si>
+  <si>
+    <t>[771, 772, 773]</t>
+  </si>
+  <si>
     <t>usa</t>
   </si>
   <si>
@@ -191,12 +197,6 @@
   </si>
   <si>
     <t>[1671, 1672]</t>
-  </si>
-  <si>
-    <t>italy</t>
-  </si>
-  <si>
-    <t>[771, 772, 773]</t>
   </si>
   <si>
     <t>germany</t>
@@ -488,10 +488,10 @@
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1037,16 +1037,16 @@
     </row>
     <row r="5">
       <c r="A5" s="5">
-        <v>167.0</v>
+        <v>77.0</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="18">
-        <v>45467.0</v>
+      <c r="C5" s="7">
+        <v>45418.0</v>
       </c>
       <c r="D5" s="8">
-        <v>219.0</v>
+        <v>358.0</v>
       </c>
       <c r="E5" s="12">
         <v>30.0</v>
@@ -1058,68 +1058,64 @@
         <v>0</v>
       </c>
       <c r="H5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="I5" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="J5" s="12">
-        <v>3.0</v>
-      </c>
-      <c r="K5" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="M5" s="12"/>
-      <c r="N5" s="20" t="s">
-        <v>29</v>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="N5" s="17" t="s">
+        <v>35</v>
       </c>
       <c r="O5" s="14">
-        <v>30.0</v>
+        <v>36.0</v>
       </c>
       <c r="P5" s="18">
-        <v>45491.0</v>
+        <v>45465.0</v>
       </c>
       <c r="Q5" s="8" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="R5" s="15">
-        <v>0.066468</v>
+        <v>0.0598</v>
       </c>
       <c r="S5" s="15">
-        <v>355.07</v>
+        <v>60.5430959723651</v>
       </c>
       <c r="T5" s="12">
-        <v>125.0</v>
+        <v>81.0</v>
       </c>
       <c r="U5" s="15">
         <f t="shared" si="1"/>
-        <v>2.84056</v>
+        <v>0.7474456293</v>
       </c>
       <c r="V5" s="15">
         <f>'Hoja 2'!$B$2*U5</f>
-        <v>0.426084</v>
+        <v>0.1121168444</v>
       </c>
       <c r="W5" s="5">
         <f>U5*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>7.625648472</v>
+        <v>2.006561249</v>
       </c>
       <c r="X5" s="21"/>
     </row>
     <row r="6">
       <c r="A6" s="5">
-        <v>77.0</v>
+        <v>167.0</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="7">
-        <v>45418.0</v>
+        <v>43</v>
+      </c>
+      <c r="C6" s="18">
+        <v>45467.0</v>
       </c>
       <c r="D6" s="8">
-        <v>358.0</v>
+        <v>27.0</v>
       </c>
       <c r="E6" s="12">
         <v>30.0</v>
@@ -1127,53 +1123,57 @@
       <c r="F6" s="11">
         <v>3.0</v>
       </c>
-      <c r="G6" s="12" t="b">
-        <v>0</v>
+      <c r="G6" s="11" t="b">
+        <v>1</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
+        <v>44</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="12">
+        <v>3.0</v>
+      </c>
       <c r="K6" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="N6" s="17" t="s">
-        <v>35</v>
+      <c r="L6" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="12"/>
+      <c r="N6" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="O6" s="14">
-        <v>36.0</v>
+        <v>20.0</v>
       </c>
       <c r="P6" s="18">
-        <v>45465.0</v>
+        <v>45494.0</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="R6" s="15">
-        <v>0.0598</v>
+        <v>0.0825</v>
       </c>
       <c r="S6" s="15">
-        <v>60.5430959723651</v>
+        <v>45.07</v>
       </c>
       <c r="T6" s="12">
-        <v>81.0</v>
+        <v>139.0</v>
       </c>
       <c r="U6" s="15">
         <f t="shared" si="1"/>
-        <v>0.7474456293</v>
+        <v>0.3242446043</v>
       </c>
       <c r="V6" s="15">
         <f>'Hoja 2'!$B$2*U6</f>
-        <v>0.1121168444</v>
+        <v>0.04863669065</v>
       </c>
       <c r="W6" s="5">
         <f>U6*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>2.006561249</v>
+        <v>0.8704534921</v>
       </c>
       <c r="X6" s="22"/>
     </row>

</xml_diff>

<commit_message>
Data italy and Germany. Reentrenando modelos.
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/df_best_models.xlsx
+++ b/main_find_best_hyper/data/df_best_models.xlsx
@@ -7,7 +7,7 @@
     <sheet state="visible" name="Hoja 2" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Hoja 1'!$A$1:$X$8</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Hoja 1'!$A$1:$Z$8</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -31,25 +31,31 @@
     </comment>
     <comment authorId="0" ref="Q1">
       <text>
-        <t xml:space="preserve">Idealmente -0.5 para que vaya por el rdo predicho (por que tal vez a la gente no le paso el resultado a apostar)</t>
+        <t xml:space="preserve">Muchas veces hay modelos outlier...
+que despues terminan cayendo y ajustandose </t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="S1">
+      <text>
+        <t xml:space="preserve">el m a utilizar cuando apuesto</t>
       </text>
     </comment>
     <comment authorId="0" ref="T1">
       <text>
+        <t xml:space="preserve">Idealmente -0.5 para que vaya por el rdo predicho (por que tal vez a la gente no le paso el resultado a apostar)</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="W1">
+      <text>
         <t xml:space="preserve">solo en las competiciones que estan en comp_to_select</t>
       </text>
     </comment>
-    <comment authorId="0" ref="V1">
+    <comment authorId="0" ref="Y1">
       <text>
         <t xml:space="preserve">usando un m=15</t>
       </text>
     </comment>
-    <comment authorId="0" ref="W1">
-      <text>
-        <t xml:space="preserve">el m a utilizar cuando apuesto</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="X2">
+    <comment authorId="0" ref="Z3">
       <text>
         <t xml:space="preserve">REVISAR DF_INTEGRATED Y VER CUAL ES LA COLUMNA QUE ES NAN Y HACE ELIMINAR PARTIDOS EN TREAT_NAN(). al sacar el fill_formaciones seguramente tenga menos registros missing. Habría que ver si rellenar con 0 “dif_val_sup” o esas que creo que son las que joden…</t>
       </text>
@@ -59,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="71">
   <si>
     <t>id_country</t>
   </si>
@@ -109,6 +115,15 @@
     <t>fecha_assess_model</t>
   </si>
   <si>
+    <t xml:space="preserve">ROI pp promedio top 10 modelos </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROI pp en partido 50 promedio top 10 modelos </t>
+  </si>
+  <si>
+    <t>m_to_use</t>
+  </si>
+  <si>
     <t>thr_prob_min_best</t>
   </si>
   <si>
@@ -127,18 +142,30 @@
     <t>ROI_por_partido realidad</t>
   </si>
   <si>
-    <t>"m" a usar</t>
-  </si>
-  <si>
     <t>Observaciones</t>
   </si>
   <si>
+    <t>france</t>
+  </si>
+  <si>
+    <t>0.8</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>[551, 552, 553, 554]</t>
+  </si>
+  <si>
+    <t>SVC</t>
+  </si>
+  <si>
+    <t>-0.15</t>
+  </si>
+  <si>
     <t>spain</t>
   </si>
   <si>
-    <t>0.8</t>
-  </si>
-  <si>
     <t>0.1</t>
   </si>
   <si>
@@ -154,22 +181,8 @@
     <t>-0.2</t>
   </si>
   <si>
-    <t>Todos los modelos de SPA tienen sesgo debido a una mala integracion. Tengo que mejorar la integracion urgentemente</t>
-  </si>
-  <si>
-    <t>france</t>
-  </si>
-  <si>
-    <t>0.2</t>
-  </si>
-  <si>
-    <t>[551, 552, 553, 554]</t>
-  </si>
-  <si>
-    <t>SVC</t>
-  </si>
-  <si>
-    <t>-0.15</t>
+    <t>Todos los modelos de SPA tienen sesgo debido a una mala integracion. Tengo que mejorar la integracion urgentemente
+Excluyo el modelo que mejor rinde porque claramente es demasiado outlier.</t>
   </si>
   <si>
     <t>england</t>
@@ -187,9 +200,20 @@
     <t>italy</t>
   </si>
   <si>
+    <t>0.7</t>
+  </si>
+  <si>
     <t>[771, 772, 773]</t>
   </si>
   <si>
+    <t>-0.1</t>
+  </si>
+  <si>
+    <t>Antes de incluir Serie B, los promedios en los top 10 modelos eran al menos tres veces mejores y en menos partidos (81 en vez de 100). Claramente la integracion tiene un gran impacto en los resultados.
+- ROI pp promedio top 10 modelos: 31,4
+- ROI pp partido 50 promedio top 10 modelos: 17,3</t>
+  </si>
+  <si>
     <t>usa</t>
   </si>
   <si>
@@ -199,10 +223,7 @@
     <t>[1671, 1672]</t>
   </si>
   <si>
-    <t>germany</t>
-  </si>
-  <si>
-    <t>[591, 593, 594]</t>
+    <t>21/7 - Paso del modelo 219 al 27 que es igual salvo que is_localia = True. Me parece correcto. A ver si este nuevo modelo tiene menos volatilidad que el 219.</t>
   </si>
   <si>
     <t>argentina</t>
@@ -320,6 +341,12 @@
     </r>
   </si>
   <si>
+    <t>germany</t>
+  </si>
+  <si>
+    <t>[591, 593, 594]</t>
+  </si>
+  <si>
     <t>Parametros para apostar</t>
   </si>
   <si>
@@ -329,19 +356,51 @@
     <t>max m</t>
   </si>
   <si>
+    <t xml:space="preserve">Promedio ROI pp top 10 modelos </t>
+  </si>
+  <si>
     <t>max roi pp</t>
+  </si>
+  <si>
+    <t>14.53</t>
+  </si>
+  <si>
+    <t>-0.46</t>
+  </si>
+  <si>
+    <t>3.40</t>
+  </si>
+  <si>
+    <t>0.29</t>
+  </si>
+  <si>
+    <t>-0.90</t>
+  </si>
+  <si>
+    <t>-0.18</t>
+  </si>
+  <si>
+    <t>4.55</t>
+  </si>
+  <si>
+    <t>-0.40</t>
+  </si>
+  <si>
+    <t>12.73</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy&quot;-&quot;mm&quot;-&quot;dd"/>
-    <numFmt numFmtId="165" formatCode="d/MM/yyyy"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="d/MM/yyyy"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="168" formatCode="dd.mm"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -372,8 +431,13 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -382,12 +446,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF9900"/>
+        <bgColor rgb="FFFF9900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8CCE4"/>
+        <bgColor rgb="FFB8CCE4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+        <bgColor rgb="FFDCE6F1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border/>
     <border>
       <top style="thin">
@@ -421,11 +509,25 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="45">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -438,6 +540,9 @@
     <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -454,74 +559,98 @@
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="3" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="3" fillId="2" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="4" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="3" fillId="2" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="4" numFmtId="167" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="9" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="10" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="9" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="5" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="6" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -741,7 +870,7 @@
   <cols>
     <col customWidth="1" min="11" max="11" width="20.5"/>
     <col customWidth="1" min="14" max="14" width="15.13"/>
-    <col customWidth="1" min="24" max="24" width="65.13"/>
+    <col customWidth="1" min="26" max="26" width="65.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -793,189 +922,207 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="V1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="Y1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="5">
+      <c r="A2" s="6">
+        <v>55.0</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="8">
+        <v>45419.0</v>
+      </c>
+      <c r="D2" s="9">
+        <v>91.0</v>
+      </c>
+      <c r="E2" s="10">
+        <v>30.0</v>
+      </c>
+      <c r="F2" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G2" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" s="13">
+        <v>18.0</v>
+      </c>
+      <c r="P2" s="14">
+        <v>45465.0</v>
+      </c>
+      <c r="Q2" s="15">
+        <v>341.17</v>
+      </c>
+      <c r="R2" s="15">
+        <v>228.32</v>
+      </c>
+      <c r="S2" s="6">
+        <f>R2*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
+        <v>30</v>
+      </c>
+      <c r="T2" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="U2" s="16">
+        <v>15.0684194244387</v>
+      </c>
+      <c r="V2" s="16">
+        <v>445.1980482158149</v>
+      </c>
+      <c r="W2" s="10">
+        <v>56.0</v>
+      </c>
+      <c r="X2" s="16">
+        <f t="shared" ref="X2:X8" si="1">V2/W2</f>
+        <v>7.949965147</v>
+      </c>
+      <c r="Y2" s="16">
+        <f>'Hoja 2'!$B$2*X2</f>
+        <v>1.192494772</v>
+      </c>
+      <c r="Z2" s="17"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6">
         <v>148.0</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="7">
+      <c r="B3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="8">
         <v>45418.0</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D3" s="9">
         <v>547.0</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E3" s="18">
         <v>60.0</v>
       </c>
-      <c r="F2" s="10">
+      <c r="F3" s="19">
         <v>3.0</v>
       </c>
-      <c r="G2" s="9" t="b">
+      <c r="G3" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11" t="s">
+      <c r="H3" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" s="11"/>
-      <c r="N2" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="O2" s="14">
-        <v>25.0</v>
-      </c>
-      <c r="P2" s="7">
-        <v>45440.0</v>
-      </c>
-      <c r="Q2" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" s="15">
-        <v>36.8495516929146</v>
-      </c>
-      <c r="S2" s="15">
-        <v>1016.9271280401779</v>
-      </c>
-      <c r="T2" s="12">
-        <v>91.0</v>
-      </c>
-      <c r="U2" s="15">
-        <f t="shared" ref="U2:U8" si="1">S2/T2</f>
-        <v>11.17502339</v>
-      </c>
-      <c r="V2" s="15">
-        <f>'Hoja 2'!$B$2*U2</f>
-        <v>1.676253508</v>
-      </c>
-      <c r="W2" s="5">
-        <f>U2*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>30</v>
-      </c>
-      <c r="X2" s="16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5">
-        <v>55.0</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="7">
-        <v>45419.0</v>
-      </c>
-      <c r="D3" s="8">
-        <v>91.0</v>
-      </c>
-      <c r="E3" s="12">
-        <v>30.0</v>
-      </c>
-      <c r="F3" s="11">
-        <v>3.0</v>
-      </c>
-      <c r="G3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="12">
-        <v>5.0</v>
-      </c>
+      <c r="J3" s="11"/>
       <c r="K3" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="11"/>
+      <c r="L3" s="10" t="s">
+        <v>35</v>
+      </c>
       <c r="M3" s="11"/>
-      <c r="N3" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3" s="14">
-        <v>18.0</v>
-      </c>
-      <c r="P3" s="18">
-        <v>45465.0</v>
-      </c>
-      <c r="Q3" s="8" t="s">
+      <c r="N3" s="20" t="s">
         <v>36</v>
       </c>
+      <c r="O3" s="13">
+        <v>25.0</v>
+      </c>
+      <c r="P3" s="8">
+        <v>45440.0</v>
+      </c>
+      <c r="Q3" s="15">
+        <v>47.49</v>
+      </c>
       <c r="R3" s="15">
-        <v>15.0684194244387</v>
-      </c>
-      <c r="S3" s="15">
-        <v>445.1980482158149</v>
-      </c>
-      <c r="T3" s="12">
-        <v>56.0</v>
-      </c>
-      <c r="U3" s="15">
+        <v>182.82</v>
+      </c>
+      <c r="S3" s="6">
+        <f>R3*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
+        <v>24.0215487</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="U3" s="16">
+        <v>36.8495516929146</v>
+      </c>
+      <c r="V3" s="16">
+        <v>1016.9271280401779</v>
+      </c>
+      <c r="W3" s="10">
+        <v>91.0</v>
+      </c>
+      <c r="X3" s="16">
         <f t="shared" si="1"/>
-        <v>7.949965147</v>
-      </c>
-      <c r="V3" s="15">
-        <f>'Hoja 2'!$B$2*U3</f>
-        <v>1.192494772</v>
-      </c>
-      <c r="W3" s="5">
-        <f>U3*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>21.34214365</v>
-      </c>
-      <c r="X3" s="19"/>
+        <v>11.17502339</v>
+      </c>
+      <c r="Y3" s="16">
+        <f>'Hoja 2'!$B$2*X3</f>
+        <v>1.676253508</v>
+      </c>
+      <c r="Z3" s="21" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>48.0</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="7">
+      <c r="B4" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="8">
         <v>45419.0</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <v>808.0</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="10">
         <v>60.0</v>
       </c>
       <c r="F4" s="11">
@@ -986,138 +1133,157 @@
       </c>
       <c r="H4" s="11"/>
       <c r="I4" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" s="12">
+        <v>28</v>
+      </c>
+      <c r="J4" s="22">
         <v>3.0</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="L4" s="12" t="s">
-        <v>28</v>
+        <v>40</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="N4" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O4" s="14">
+        <v>41</v>
+      </c>
+      <c r="N4" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="O4" s="13">
         <v>34.0</v>
       </c>
-      <c r="P4" s="18">
+      <c r="P4" s="14">
         <v>45465.0</v>
       </c>
-      <c r="Q4" s="5" t="s">
-        <v>40</v>
+      <c r="Q4" s="15">
+        <v>55.29</v>
       </c>
       <c r="R4" s="15">
+        <v>17.63</v>
+      </c>
+      <c r="S4" s="6">
+        <f>R4*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
+        <v>2.316485634</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="U4" s="16">
         <v>0.52</v>
       </c>
-      <c r="S4" s="15">
+      <c r="V4" s="16">
         <v>526.3246948871299</v>
       </c>
-      <c r="T4" s="11">
+      <c r="W4" s="11">
         <v>122.0</v>
       </c>
-      <c r="U4" s="15">
+      <c r="X4" s="16">
         <f t="shared" si="1"/>
         <v>4.314136843</v>
       </c>
-      <c r="V4" s="15">
-        <f>'Hoja 2'!$B$2*U4</f>
+      <c r="Y4" s="16">
+        <f>'Hoja 2'!$B$2*X4</f>
         <v>0.6471205265</v>
       </c>
-      <c r="W4" s="5">
-        <f>U4*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>11.58155118</v>
-      </c>
-      <c r="X4" s="19"/>
+      <c r="Z4" s="17"/>
     </row>
     <row r="5">
-      <c r="A5" s="5">
+      <c r="A5" s="6">
         <v>77.0</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="7">
-        <v>45418.0</v>
-      </c>
-      <c r="D5" s="8">
-        <v>358.0</v>
-      </c>
-      <c r="E5" s="12">
+      <c r="B5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="14">
+        <v>45497.0</v>
+      </c>
+      <c r="D5" s="9">
+        <v>194.0</v>
+      </c>
+      <c r="E5" s="10">
         <v>30.0</v>
       </c>
       <c r="F5" s="11">
         <v>3.0</v>
       </c>
-      <c r="G5" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
+      <c r="G5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" s="10">
+        <v>10.0</v>
+      </c>
       <c r="K5" s="11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="L5" s="11"/>
       <c r="M5" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="N5" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O5" s="14">
-        <v>36.0</v>
-      </c>
-      <c r="P5" s="18">
+        <v>41</v>
+      </c>
+      <c r="N5" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O5" s="13">
+        <v>11.0</v>
+      </c>
+      <c r="P5" s="14">
         <v>45465.0</v>
       </c>
-      <c r="Q5" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="R5" s="15">
-        <v>0.0598</v>
-      </c>
-      <c r="S5" s="15">
-        <v>60.5430959723651</v>
-      </c>
-      <c r="T5" s="12">
-        <v>81.0</v>
-      </c>
-      <c r="U5" s="15">
+      <c r="Q5" s="24">
+        <v>15.508000000000001</v>
+      </c>
+      <c r="R5" s="25">
+        <v>3.97</v>
+      </c>
+      <c r="S5" s="6">
+        <f>R5*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
+        <v>0.5216362999</v>
+      </c>
+      <c r="T5" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="U5" s="26">
+        <v>0.1452</v>
+      </c>
+      <c r="V5" s="16">
+        <v>48.05</v>
+      </c>
+      <c r="W5" s="10">
+        <v>100.0</v>
+      </c>
+      <c r="X5" s="16">
         <f t="shared" si="1"/>
-        <v>0.7474456293</v>
-      </c>
-      <c r="V5" s="15">
-        <f>'Hoja 2'!$B$2*U5</f>
-        <v>0.1121168444</v>
-      </c>
-      <c r="W5" s="5">
-        <f>U5*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>2.006561249</v>
-      </c>
-      <c r="X5" s="21"/>
+        <v>0.4805</v>
+      </c>
+      <c r="Y5" s="16">
+        <f>'Hoja 2'!$B$2*X5</f>
+        <v>0.072075</v>
+      </c>
+      <c r="Z5" s="27" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD5" s="28"/>
     </row>
     <row r="6">
-      <c r="A6" s="5">
+      <c r="A6" s="6">
         <v>167.0</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="18">
+      <c r="B6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="14">
         <v>45467.0</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <v>27.0</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="10">
         <v>30.0</v>
       </c>
       <c r="F6" s="11">
@@ -1126,72 +1292,81 @@
       <c r="G6" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="H6" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="12">
+      <c r="H6" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="22">
         <v>3.0</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="L6" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="M6" s="12"/>
-      <c r="N6" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="O6" s="14">
+        <v>50</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="M6" s="10"/>
+      <c r="N6" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="O6" s="13">
         <v>20.0</v>
       </c>
-      <c r="P6" s="18">
+      <c r="P6" s="14">
         <v>45494.0</v>
       </c>
-      <c r="Q6" s="8" t="s">
-        <v>40</v>
+      <c r="Q6" s="15">
+        <v>17.23</v>
       </c>
       <c r="R6" s="15">
+        <v>3.59</v>
+      </c>
+      <c r="S6" s="6">
+        <f>R6*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
+        <v>0.471706377</v>
+      </c>
+      <c r="T6" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="U6" s="16">
         <v>0.0825</v>
       </c>
-      <c r="S6" s="15">
+      <c r="V6" s="16">
         <v>45.07</v>
       </c>
-      <c r="T6" s="12">
+      <c r="W6" s="10">
         <v>139.0</v>
       </c>
-      <c r="U6" s="15">
+      <c r="X6" s="16">
         <f t="shared" si="1"/>
         <v>0.3242446043</v>
       </c>
-      <c r="V6" s="15">
-        <f>'Hoja 2'!$B$2*U6</f>
+      <c r="Y6" s="16">
+        <f>'Hoja 2'!$B$2*X6</f>
         <v>0.04863669065</v>
       </c>
-      <c r="W6" s="5">
-        <f>U6*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>0.8704534921</v>
-      </c>
-      <c r="X6" s="22"/>
+      <c r="Z6" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD6" s="29"/>
     </row>
     <row r="7">
-      <c r="A7" s="5">
-        <v>59.0</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="7">
-        <v>45421.0</v>
-      </c>
-      <c r="D7" s="5">
-        <v>1757.0</v>
+      <c r="A7" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="8">
+        <v>45419.0</v>
+      </c>
+      <c r="D7" s="9">
+        <v>779.0</v>
       </c>
       <c r="E7" s="11">
-        <v>60.0</v>
+        <v>30.0</v>
       </c>
       <c r="F7" s="11">
         <v>3.0</v>
@@ -1199,162 +1374,189 @@
       <c r="G7" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="J7" s="11">
+      <c r="H7" s="11"/>
+      <c r="I7" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J7" s="10">
+        <v>10.0</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="O7" s="13">
+        <v>21.0</v>
+      </c>
+      <c r="P7" s="14">
+        <v>45488.0</v>
+      </c>
+      <c r="Q7" s="15">
+        <v>8.402</v>
+      </c>
+      <c r="R7" s="15">
+        <v>3.56</v>
+      </c>
+      <c r="S7" s="6">
+        <f>R7*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
+        <v>0.467764541</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="U7" s="26">
+        <v>-6.0E-4</v>
+      </c>
+      <c r="V7" s="16">
+        <v>8.39</v>
+      </c>
+      <c r="W7" s="10">
+        <v>92.0</v>
+      </c>
+      <c r="X7" s="16">
+        <f t="shared" si="1"/>
+        <v>0.09119565217</v>
+      </c>
+      <c r="Y7" s="16">
+        <f>'Hoja 2'!$B$2*X7</f>
+        <v>0.01367934783</v>
+      </c>
+      <c r="Z7" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD7" s="29"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6">
+        <v>59.0</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="8">
+        <v>45421.0</v>
+      </c>
+      <c r="D8" s="6">
+        <v>1757.0</v>
+      </c>
+      <c r="E8" s="11">
+        <v>60.0</v>
+      </c>
+      <c r="F8" s="11">
         <v>3.0</v>
       </c>
-      <c r="K7" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="L7" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="M7" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="N7" s="17" t="s">
+      <c r="G8" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J8" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L8" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="O7" s="14">
+      <c r="M8" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O8" s="13">
         <v>32.0</v>
       </c>
-      <c r="P7" s="18">
+      <c r="P8" s="14">
         <v>45465.0</v>
       </c>
-      <c r="Q7" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="R7" s="23"/>
-      <c r="S7" s="15">
+      <c r="Q8" s="30"/>
+      <c r="R8" s="30"/>
+      <c r="S8" s="6">
+        <f>R8*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
+        <v>0</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="U8" s="31"/>
+      <c r="V8" s="16">
         <v>4.0</v>
       </c>
-      <c r="T7" s="12">
+      <c r="W8" s="10">
         <v>20.0</v>
       </c>
-      <c r="U7" s="15">
+      <c r="X8" s="16">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="V7" s="15">
-        <f>'Hoja 2'!$B$2*U7</f>
+      <c r="Y8" s="16">
+        <f>'Hoja 2'!$B$2*X8</f>
         <v>0.03</v>
       </c>
-      <c r="W7" s="5">
-        <f>U7*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>0.5369116281</v>
-      </c>
-      <c r="X7" s="19"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5">
-        <v>6.0</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="7">
-        <v>45419.0</v>
-      </c>
-      <c r="D8" s="8">
-        <v>779.0</v>
-      </c>
-      <c r="E8" s="11">
-        <v>30.0</v>
-      </c>
-      <c r="F8" s="11">
-        <v>3.0</v>
-      </c>
-      <c r="G8" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="H8" s="11"/>
-      <c r="I8" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="J8" s="12">
-        <v>10.0</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="L8" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="M8" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="N8" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="O8" s="14">
-        <v>21.0</v>
-      </c>
-      <c r="P8" s="18">
-        <v>45488.0</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="R8" s="24">
-        <v>-6.0E-4</v>
-      </c>
-      <c r="S8" s="15">
-        <v>8.39</v>
-      </c>
-      <c r="T8" s="12">
-        <v>92.0</v>
-      </c>
-      <c r="U8" s="15">
-        <f t="shared" si="1"/>
-        <v>0.09119565217</v>
-      </c>
-      <c r="V8" s="15">
-        <f>'Hoja 2'!$B$2*U8</f>
-        <v>0.01367934783</v>
-      </c>
-      <c r="W8" s="5">
-        <f>U8*'Hoja 2'!$B$3/'Hoja 2'!$B$4</f>
-        <v>0.2448200304</v>
-      </c>
-      <c r="X8" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z8" s="26"/>
-      <c r="AA8" s="26"/>
+      <c r="Z8" s="17"/>
+      <c r="AD8" s="29"/>
+    </row>
+    <row r="9">
+      <c r="AD9" s="29"/>
     </row>
     <row r="10">
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="F10" s="28"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="F10" s="33"/>
+      <c r="Y10" s="34"/>
+      <c r="AD10" s="29"/>
     </row>
     <row r="11">
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="W11" s="29"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="Q11" s="35"/>
+      <c r="R11" s="35"/>
+      <c r="S11" s="35"/>
+      <c r="AD11" s="29"/>
     </row>
     <row r="12">
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="Q12" s="28"/>
+      <c r="R12" s="36"/>
+      <c r="AD12" s="29"/>
     </row>
     <row r="13">
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="R13" s="36"/>
+      <c r="Y13" s="35"/>
+      <c r="AD13" s="29"/>
+    </row>
+    <row r="14">
+      <c r="R14" s="35"/>
+      <c r="AD14" s="29"/>
     </row>
     <row r="17">
-      <c r="H17" s="28"/>
+      <c r="H17" s="33"/>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$X$8">
-    <sortState ref="A1:X8">
-      <sortCondition descending="1" ref="U1:U8"/>
+  <autoFilter ref="$A$1:$Z$8">
+    <sortState ref="A1:Z8">
+      <sortCondition descending="1" ref="R1:R8"/>
+      <sortCondition descending="1" ref="X1:X8"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="T2:T8">
+  <conditionalFormatting sqref="W2:W8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1364,7 +1566,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:V8">
+  <conditionalFormatting sqref="X2:Y8">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1374,7 +1576,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S8">
+  <conditionalFormatting sqref="V2:V8">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1397,41 +1599,136 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="30" t="s">
-        <v>51</v>
+      <c r="A1" s="37" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" s="32">
+      <c r="A2" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="39">
         <v>0.15</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="31">
+      <c r="A3" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="38">
         <v>30.0</v>
       </c>
+      <c r="E3" s="38" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="33">
-        <f>MAX('Hoja 1'!U2:U8)</f>
-        <v>11.17502339</v>
+      <c r="A4" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="40">
+        <f>MAX('Hoja 1'!R2:R8)</f>
+        <v>228.32</v>
+      </c>
+      <c r="F4" s="29">
+        <f>AVERAGE(F7:F16)</f>
+        <v>3.965</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26">
+      <c r="A7" s="41">
         <v>30.0</v>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="41">
         <v>1118.0</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" s="29">
+        <f t="shared" ref="F7:F16" si="1">REPLACE(E7,FIND(".",E7),1,",")*1</f>
+        <v>14.53</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="E8" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" s="29">
+        <f t="shared" si="1"/>
+        <v>-0.46</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="E9" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="29">
+        <f t="shared" si="1"/>
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="E10" s="44">
+        <v>45541.0</v>
+      </c>
+      <c r="F10" s="29">
+        <f t="shared" si="1"/>
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="E11" s="42" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" s="29">
+        <f t="shared" si="1"/>
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="F12" s="29">
+        <f t="shared" si="1"/>
+        <v>-0.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="E13" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="F13" s="29">
+        <f t="shared" si="1"/>
+        <v>-0.18</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="29">
+        <f t="shared" si="1"/>
+        <v>4.55</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="F15" s="29">
+        <f t="shared" si="1"/>
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="29">
+        <f t="shared" si="1"/>
+        <v>12.73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>